<commit_message>
feat: Remove attribute-level up-to-date details from xlsx template
[#OCD-4888]
</commit_message>
<xml_diff>
--- a/chpl/chpl-resources/src/main/resources/UpdatedCriteriaStatusReport.xlsx
+++ b/chpl/chpl-resources/src/main/resources/UpdatedCriteriaStatusReport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\youngto\workspaces\chpladmin\chpl-api\chpl\chpl-resources\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekeyk\projects\chpl-api\chpl\chpl-resources\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45C9C060-2115-4814-966F-30DE69EB4DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54FD02D2-E832-444C-A0DD-C6182E444C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{68FE7958-BC57-49F5-AC1F-F5C1A57C91FE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{68FE7958-BC57-49F5-AC1F-F5C1A57C91FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="11" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Requires Update</t>
   </si>
@@ -45,16 +45,7 @@
     <t>Fully Up-to-Date</t>
   </si>
   <si>
-    <t>Standards Up-to-Date</t>
-  </si>
-  <si>
-    <t>Code Sets Up-to-Date</t>
-  </si>
-  <si>
     <t>Total listings for criterion</t>
-  </si>
-  <si>
-    <t>Functionalities Tested Up-to-Date</t>
   </si>
 </sst>
 </file>
@@ -458,7 +449,7 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Template!$B$7:$M$7</c:f>
+              <c:f>Template!$B$4:$M$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -505,234 +496,6 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-B3A1-4AB1-AF38-4762E76F6310}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="4"/>
-          <c:order val="5"/>
-          <c:tx>
-            <c:v>Code Sets Up-to-Date</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="diamond"/>
-            <c:size val="7"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:sysClr val="window" lastClr="FFFFFF"/>
-              </a:solidFill>
-            </c:spPr>
-          </c:marker>
-          <c:val>
-            <c:numRef>
-              <c:f>Template!$B$4:$M$4</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-B3A1-4AB1-AF38-4762E76F6310}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="5"/>
-          <c:order val="6"/>
-          <c:tx>
-            <c:v>Functionality Up-to-Date</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:srgbClr val="00B0F0"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="diamond"/>
-            <c:size val="7"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:sysClr val="window" lastClr="FFFFFF"/>
-              </a:solidFill>
-            </c:spPr>
-          </c:marker>
-          <c:val>
-            <c:numRef>
-              <c:f>Template!$B$5:$M$5</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-B3A1-4AB1-AF38-4762E76F6310}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="7"/>
-          <c:order val="7"/>
-          <c:tx>
-            <c:v>Standards Up-to-Date</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="diamond"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-            </c:spPr>
-          </c:marker>
-          <c:val>
-            <c:numRef>
-              <c:f>Template!$B$6:$M$6</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-B3A1-4AB1-AF38-4762E76F6310}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1003,6 +766,132 @@
                 <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000007-B3A1-4AB1-AF38-4762E76F6310}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredLineSeries>
+            <c15:filteredLineSeries>
+              <c15:ser>
+                <c:idx val="4"/>
+                <c:order val="5"/>
+                <c:tx>
+                  <c:v>Code Sets Up-to-Date</c:v>
+                </c:tx>
+                <c:marker>
+                  <c:symbol val="diamond"/>
+                  <c:size val="7"/>
+                  <c:spPr>
+                    <a:solidFill>
+                      <a:sysClr val="window" lastClr="FFFFFF"/>
+                    </a:solidFill>
+                  </c:spPr>
+                </c:marker>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Template!#REF!</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>1</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000003-B3A1-4AB1-AF38-4762E76F6310}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredLineSeries>
+            <c15:filteredLineSeries>
+              <c15:ser>
+                <c:idx val="5"/>
+                <c:order val="6"/>
+                <c:tx>
+                  <c:v>Functionality Up-to-Date</c:v>
+                </c:tx>
+                <c:marker>
+                  <c:symbol val="diamond"/>
+                  <c:size val="7"/>
+                  <c:spPr>
+                    <a:solidFill>
+                      <a:sysClr val="window" lastClr="FFFFFF"/>
+                    </a:solidFill>
+                  </c:spPr>
+                </c:marker>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Template!#REF!</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>1</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000004-B3A1-4AB1-AF38-4762E76F6310}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredLineSeries>
+            <c15:filteredLineSeries>
+              <c15:ser>
+                <c:idx val="7"/>
+                <c:order val="7"/>
+                <c:tx>
+                  <c:v>Standards Up-to-Date</c:v>
+                </c:tx>
+                <c:marker>
+                  <c:symbol val="diamond"/>
+                  <c:size val="5"/>
+                  <c:spPr>
+                    <a:solidFill>
+                      <a:schemeClr val="bg1"/>
+                    </a:solidFill>
+                  </c:spPr>
+                </c:marker>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Template!#REF!</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>1</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000005-B3A1-4AB1-AF38-4762E76F6310}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -1213,13 +1102,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>546100</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>68580</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1547,14 +1436,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04F5CA64-B349-4540-8897-9876CE15B639}">
-  <dimension ref="A1:U8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:U5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="31.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1595,60 +1484,60 @@
         <v>45349</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2">
-        <f t="shared" ref="B2:M2" si="0">B7-B3</f>
+        <f>B4-B3</f>
         <v>0</v>
       </c>
       <c r="C2">
-        <f t="shared" si="0"/>
+        <f>C4-C3</f>
         <v>0</v>
       </c>
       <c r="D2">
-        <f t="shared" si="0"/>
+        <f>D4-D3</f>
         <v>0</v>
       </c>
       <c r="E2">
-        <f t="shared" si="0"/>
+        <f>E4-E3</f>
         <v>0</v>
       </c>
       <c r="F2">
-        <f t="shared" si="0"/>
+        <f>F4-F3</f>
         <v>0</v>
       </c>
       <c r="G2">
-        <f t="shared" si="0"/>
+        <f>G4-G3</f>
         <v>0</v>
       </c>
       <c r="H2">
-        <f t="shared" si="0"/>
+        <f>H4-H3</f>
         <v>0</v>
       </c>
       <c r="I2">
-        <f t="shared" si="0"/>
+        <f>I4-I3</f>
         <v>0</v>
       </c>
       <c r="J2">
-        <f t="shared" si="0"/>
+        <f>J4-J3</f>
         <v>0</v>
       </c>
       <c r="K2">
-        <f t="shared" si="0"/>
+        <f>K4-K3</f>
         <v>0</v>
       </c>
       <c r="L2">
-        <f t="shared" si="0"/>
+        <f>L4-L3</f>
         <v>0</v>
       </c>
       <c r="M2">
-        <f t="shared" si="0"/>
+        <f>M4-M3</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1689,9 +1578,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1729,146 +1618,21 @@
       <c r="M4">
         <v>0</v>
       </c>
+      <c r="U4" s="3"/>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="U5" s="3"/>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="U6" s="3"/>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="U7" s="3"/>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1877,6 +1641,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100054B99873F0D6546B559819D0825E003" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cffa56ad5792ecafcd3589bab1bbb308">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="63b9e3fc-e3d9-4b25-9f08-bf71a160189f" xmlns:ns4="6c1397f4-a2e4-41e1-a56a-3ef30e67d471" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68c1c6e3f17b441c567360df559ac01a" ns3:_="" ns4:_="">
     <xsd:import namespace="63b9e3fc-e3d9-4b25-9f08-bf71a160189f"/>
@@ -2115,15 +1888,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2133,6 +1897,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30F5C5E2-FF74-4F0D-A48F-2A211F06009F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBA91FC1-FB23-421D-B0F5-8B5FD962DF28}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2147,14 +1919,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30F5C5E2-FF74-4F0D-A48F-2A211F06009F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
refactor: Pull out report date calculation to a service
[#OCD-4888]
</commit_message>
<xml_diff>
--- a/chpl/chpl-resources/src/main/resources/UpdatedCriteriaStatusReport.xlsx
+++ b/chpl/chpl-resources/src/main/resources/UpdatedCriteriaStatusReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekeyk\projects\chpl-api\chpl\chpl-resources\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54FD02D2-E832-444C-A0DD-C6182E444C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C52486E5-5726-4D9B-B08C-8E7484A6DED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{68FE7958-BC57-49F5-AC1F-F5C1A57C91FE}"/>
   </bookViews>
@@ -511,393 +511,7 @@
         <c:smooth val="0"/>
         <c:axId val="697930415"/>
         <c:axId val="697937487"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredLineSeries>
-              <c15:ser>
-                <c:idx val="3"/>
-                <c:order val="3"/>
-                <c:tx>
-                  <c:v>% Fully Up-to-Date</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent1"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="circle"/>
-                  <c:size val="5"/>
-                  <c:spPr>
-                    <a:solidFill>
-                      <a:schemeClr val="accent1"/>
-                    </a:solidFill>
-                    <a:ln w="9525">
-                      <a:solidFill>
-                        <a:schemeClr val="accent1"/>
-                      </a:solidFill>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c:marker>
-                <c:dLbls>
-                  <c:spPr>
-                    <a:noFill/>
-                    <a:ln>
-                      <a:noFill/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                  <c:txPr>
-                    <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                      <a:spAutoFit/>
-                    </a:bodyPr>
-                    <a:lstStyle/>
-                    <a:p>
-                      <a:pPr>
-                        <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                          <a:solidFill>
-                            <a:schemeClr val="tx1">
-                              <a:lumMod val="75000"/>
-                              <a:lumOff val="25000"/>
-                            </a:schemeClr>
-                          </a:solidFill>
-                          <a:latin typeface="+mn-lt"/>
-                          <a:ea typeface="+mn-ea"/>
-                          <a:cs typeface="+mn-cs"/>
-                        </a:defRPr>
-                      </a:pPr>
-                      <a:endParaRPr lang="en-US"/>
-                    </a:p>
-                  </c:txPr>
-                  <c:dLblPos val="t"/>
-                  <c:showLegendKey val="0"/>
-                  <c:showVal val="1"/>
-                  <c:showCatName val="0"/>
-                  <c:showSerName val="0"/>
-                  <c:showPercent val="0"/>
-                  <c:showBubbleSize val="0"/>
-                  <c:showLeaderLines val="0"/>
-                  <c:extLst>
-                    <c:ext uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                      <c15:showLeaderLines val="0"/>
-                    </c:ext>
-                  </c:extLst>
-                </c:dLbls>
-                <c:cat>
-                  <c:numLit>
-                    <c:formatCode>General</c:formatCode>
-                    <c:ptCount val="12"/>
-                    <c:pt idx="0">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="1">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="2">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="3">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="4">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="5">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="6">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="7">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="8">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="9">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="10">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="11">
-                      <c:v>0</c:v>
-                    </c:pt>
-                  </c:numLit>
-                </c:cat>
-                <c:val>
-                  <c:numLit>
-                    <c:formatCode>General</c:formatCode>
-                    <c:ptCount val="12"/>
-                    <c:pt idx="0">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="1">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="2">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="3">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="4">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="5">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="6">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="7">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="8">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="9">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="10">
-                      <c:v>0</c:v>
-                    </c:pt>
-                    <c:pt idx="11">
-                      <c:v>0</c:v>
-                    </c:pt>
-                  </c:numLit>
-                </c:val>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000006-B3A1-4AB1-AF38-4762E76F6310}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredLineSeries>
-            <c15:filteredLineSeries>
-              <c15:ser>
-                <c:idx val="2"/>
-                <c:order val="4"/>
-                <c:tx>
-                  <c:v>Fully Up-to-Date</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent1"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="circle"/>
-                  <c:size val="5"/>
-                  <c:spPr>
-                    <a:solidFill>
-                      <a:schemeClr val="accent3"/>
-                    </a:solidFill>
-                    <a:ln w="9525">
-                      <a:solidFill>
-                        <a:schemeClr val="accent1"/>
-                      </a:solidFill>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c:marker>
-                <c:val>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Template!$B$3:$M$3</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="12"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="5">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="6">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="7">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="8">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="9">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="10">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="11">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:val>
-                <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000007-B3A1-4AB1-AF38-4762E76F6310}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredLineSeries>
-            <c15:filteredLineSeries>
-              <c15:ser>
-                <c:idx val="4"/>
-                <c:order val="5"/>
-                <c:tx>
-                  <c:v>Code Sets Up-to-Date</c:v>
-                </c:tx>
-                <c:marker>
-                  <c:symbol val="diamond"/>
-                  <c:size val="7"/>
-                  <c:spPr>
-                    <a:solidFill>
-                      <a:sysClr val="window" lastClr="FFFFFF"/>
-                    </a:solidFill>
-                  </c:spPr>
-                </c:marker>
-                <c:val>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Template!#REF!</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>1</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:val>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000003-B3A1-4AB1-AF38-4762E76F6310}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredLineSeries>
-            <c15:filteredLineSeries>
-              <c15:ser>
-                <c:idx val="5"/>
-                <c:order val="6"/>
-                <c:tx>
-                  <c:v>Functionality Up-to-Date</c:v>
-                </c:tx>
-                <c:marker>
-                  <c:symbol val="diamond"/>
-                  <c:size val="7"/>
-                  <c:spPr>
-                    <a:solidFill>
-                      <a:sysClr val="window" lastClr="FFFFFF"/>
-                    </a:solidFill>
-                  </c:spPr>
-                </c:marker>
-                <c:val>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Template!#REF!</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>1</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:val>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000004-B3A1-4AB1-AF38-4762E76F6310}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredLineSeries>
-            <c15:filteredLineSeries>
-              <c15:ser>
-                <c:idx val="7"/>
-                <c:order val="7"/>
-                <c:tx>
-                  <c:v>Standards Up-to-Date</c:v>
-                </c:tx>
-                <c:marker>
-                  <c:symbol val="diamond"/>
-                  <c:size val="5"/>
-                  <c:spPr>
-                    <a:solidFill>
-                      <a:schemeClr val="bg1"/>
-                    </a:solidFill>
-                  </c:spPr>
-                </c:marker>
-                <c:val>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Template!#REF!</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>1</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:val>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000005-B3A1-4AB1-AF38-4762E76F6310}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredLineSeries>
-          </c:ext>
-        </c:extLst>
+        <c:extLst/>
       </c:lineChart>
       <c:dateAx>
         <c:axId val="697930415"/>
@@ -1489,51 +1103,39 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <f>B4-B3</f>
         <v>0</v>
       </c>
       <c r="C2">
-        <f>C4-C3</f>
         <v>0</v>
       </c>
       <c r="D2">
-        <f>D4-D3</f>
         <v>0</v>
       </c>
       <c r="E2">
-        <f>E4-E3</f>
         <v>0</v>
       </c>
       <c r="F2">
-        <f>F4-F3</f>
         <v>0</v>
       </c>
       <c r="G2">
-        <f>G4-G3</f>
         <v>0</v>
       </c>
       <c r="H2">
-        <f>H4-H3</f>
         <v>0</v>
       </c>
       <c r="I2">
-        <f>I4-I3</f>
         <v>0</v>
       </c>
       <c r="J2">
-        <f>J4-J3</f>
         <v>0</v>
       </c>
       <c r="K2">
-        <f>K4-K3</f>
         <v>0</v>
       </c>
       <c r="L2">
-        <f>L4-L3</f>
         <v>0</v>
       </c>
       <c r="M2">
-        <f>M4-M3</f>
         <v>0</v>
       </c>
     </row>
@@ -1542,39 +1144,51 @@
         <v>2</v>
       </c>
       <c r="B3">
+        <f>B4-B2</f>
         <v>0</v>
       </c>
       <c r="C3">
+        <f>C4-C2</f>
         <v>0</v>
       </c>
       <c r="D3">
+        <f t="shared" ref="D3:M3" si="0">D4-D2</f>
         <v>0</v>
       </c>
       <c r="E3">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F3">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G3">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H3">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I3">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J3">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="K3">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L3">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M3">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -1641,15 +1255,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100054B99873F0D6546B559819D0825E003" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cffa56ad5792ecafcd3589bab1bbb308">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="63b9e3fc-e3d9-4b25-9f08-bf71a160189f" xmlns:ns4="6c1397f4-a2e4-41e1-a56a-3ef30e67d471" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68c1c6e3f17b441c567360df559ac01a" ns3:_="" ns4:_="">
     <xsd:import namespace="63b9e3fc-e3d9-4b25-9f08-bf71a160189f"/>
@@ -1888,6 +1493,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1897,14 +1511,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30F5C5E2-FF74-4F0D-A48F-2A211F06009F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBA91FC1-FB23-421D-B0F5-8B5FD962DF28}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1919,6 +1525,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30F5C5E2-FF74-4F0D-A48F-2A211F06009F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>